<commit_message>
Drive Observe hazard results from import copy and stop tab publish from renaming the lesson.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10821"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37BC245B-F4E1-0040-8540-A9D3042BA5A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24FB25F2-7ACD-934D-B702-5AEEBA2BE0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-9160" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1260" yWindow="720" windowWidth="30240" windowHeight="19000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lesson" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="128">
   <si>
     <t>key</t>
   </si>
@@ -56,12 +56,6 @@
     <t>instruction</t>
   </si>
   <si>
-    <t>Scan from left to right by swiping your finger and tap the most dangerous hazards as soon as you spot it. 
-- You have 3 attempts
-- Points deducted for incorrect attempts
-- You only have 10 seconds</t>
-  </si>
-  <si>
     <t>instruction_pill</t>
   </si>
   <si>
@@ -113,9 +107,6 @@
     <t>second_instruction</t>
   </si>
   <si>
-    <t>Here are the instructions for the coaching lesson in the Observe section. We have room for quite a bit of text, but not a ton.</t>
-  </si>
-  <si>
     <t>second_instruction_pill</t>
   </si>
   <si>
@@ -245,9 +236,6 @@
     <t xml:space="preserve">Here we explain the correct answer whenever the user gets it wrong. It can be kind of long. </t>
   </si>
   <si>
-    <t>Here is a correct answer</t>
-  </si>
-  <si>
     <t>Here is a long incorrect answer that will definitely wrap into two lines</t>
   </si>
   <si>
@@ -356,17 +344,73 @@
     <t>language</t>
   </si>
   <si>
-    <t>This is a sample of the inroads MVP in french</t>
-  </si>
-  <si>
     <t>English</t>
+  </si>
+  <si>
+    <t>Canadian English inroads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You got it on your second attempt. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">You found it, but it took 3 attempts. </t>
+  </si>
+  <si>
+    <t>2_attempts</t>
+  </si>
+  <si>
+    <t>3_attempts</t>
+  </si>
+  <si>
+    <t>time_out</t>
+  </si>
+  <si>
+    <t>missed_2_attempts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You attempted once, but time ran out before you found it. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time ran out before you attempted anything. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">You tried twice and time ran out. </t>
+  </si>
+  <si>
+    <t>Let's sharpen a couple of perception skills that can help keep you safe.</t>
+  </si>
+  <si>
+    <t>success_result</t>
+  </si>
+  <si>
+    <t>NO COACHING NEEDED</t>
+  </si>
+  <si>
+    <t>fail_screen</t>
+  </si>
+  <si>
+    <t>COACHING REQUIRED</t>
+  </si>
+  <si>
+    <t>missed_1_attempt</t>
+  </si>
+  <si>
+    <t>You're about to watch a short driving video.
+Somewhere in the scenario is the primary hazard.It could be in front, behind or to either side, so drag the screen from side to side to scan the road and your mirrors.
+As soon as you spot it, click on it. You'll have a few seconds and up to three attempts. There's no replay, so watch closely. Ready? Here we go.</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Here is a kind of long correct answer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,13 +424,38 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -398,17 +467,35 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -774,7 +861,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
@@ -787,18 +874,18 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -809,7 +896,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -828,227 +915,305 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" ht="154" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="C3" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="C4" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C18" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C21" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="B22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C27" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" t="s">
-        <v>39</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -1078,61 +1243,61 @@
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
@@ -1143,1856 +1308,1856 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N2">
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="J3">
         <v>10</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>76</v>
+        <v>127</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="N4">
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="N5">
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N6">
         <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="N7">
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="N8">
         <v>0</v>
       </c>
       <c r="O8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="N9">
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N10">
         <v>0</v>
       </c>
       <c r="O10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="R31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="S31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="T31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3014,321 +3179,321 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" t="s">
         <v>97</v>
       </c>
-      <c r="B7" t="s">
-        <v>100</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
         <v>105</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B25" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>